<commit_message>
Update research integrity tracker: Frontiers Aug 2025 purge
Restore the fuller retractions data into the master and re-sync:
- split the bulk paper-mill category into Hindawi/Wiley (2021-2025, ongoing)
  and a new Frontiers RIA purge row (large batch retracted Aug 2025)
- refresh the "Key finding" note (more flagship journals listed; re-checked
  Jun 2026). Fixed at the private master so future syncs keep it.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/xlsx/research_integrity.xlsx
+++ b/data/xlsx/research_integrity.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retractions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Predatory &amp; questionable" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to maintain" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Retractions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Predatory &amp; questionable" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="How to maintain" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Retractions'!$A$1:$H$5</definedName>
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -688,22 +688,64 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>2021-2023</t>
+          <t>2021-2025</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>2022-2024</t>
+          <t>2022-2025</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>'Systematic manipulation of the publication process' — paper-mill / peer-review manipulation. Part of the industry-wide Hindawi purge (8,000+ retractions in 2023).</t>
+          <t>'Systematic manipulation of the publication process' — paper-mill / peer-review manipulation. Part of the industry-wide Hindawi purge (8,000+ retractions in 2023). Activity is ongoing, not historical.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
           <t>retractionwatch.com/category/by-publisher/hindawi/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BULK CATEGORY: 'music education / vocational music / psychology'-themed papers caught in the Frontiers integrity purge</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>various</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Frontiers in Psychology (NOT music-ed journals)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Frontiers</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2021-2024</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2024-2025</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Frontiers Research Integrity Auditing (RIA) team: peer-review with undisclosed conflicts of interest and citation manipulation; loss of confidence in findings (COPE). Large batch retracted 7 Aug 2025.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>frontiersin.org/journals/psychology (RIA retraction notices, Aug 2025)</t>
         </is>
       </c>
     </row>
@@ -929,7 +971,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Flagship journals are essentially clean (one exception: Guéguen, Psychology of Music, 2020). No sourced retractions found in MER, IJME, JRME, Musicae Scientiae, CRME, BJME. The large 'music-education-themed' cluster sits in GENERAL engineering/computing journals (Hindawi/Wiley special issues), not music-ed journals — track as one category.</t>
+          <t>Flagship music-ed journals remain essentially clean: the one sourced retraction is Guéguen, Psychology of Music (2014, retracted 2020). No sourced retractions in MER, IJME, JRME, Musicae Scientiae, CRME, BJME, RSME, JMTE, or Update. The large 'music-education-themed' cluster sits in GENERAL psychology/engineering journals (Hindawi/Wiley special issues and Frontiers in Psychology), not music-ed journals — tracked as bulk categories. This activity is ONGOING: Frontiers ran a further integrity purge in Aug 2025. Re-checked Jun 2026.</t>
         </is>
       </c>
     </row>

</xml_diff>